<commit_message>
recalc_result.xlsx 재생성 (AI 추정원인 컬럼 반영)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/recalc_result.xlsx
+++ b/recalc_result.xlsx
@@ -9,10 +9,11 @@
   <sheets>
     <sheet name="재계산결과" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="차이자산" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="유의한차이자산" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'재계산결과'!$A$1:$R$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'차이자산'!$A$1:$R$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'재계산결과'!$A$1:$T$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'차이자산'!$A$1:$T$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -444,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R14"/>
+  <dimension ref="A1:T14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -465,6 +466,8 @@
     <col width="15" customWidth="1" min="16" max="16"/>
     <col width="16" customWidth="1" min="17" max="17"/>
     <col width="14" customWidth="1" min="18" max="18"/>
+    <col width="14" customWidth="1" min="19" max="19"/>
+    <col width="60" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -556,6 +559,16 @@
       <c r="R1" s="1" t="inlineStr">
         <is>
           <t>일치여부</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>중요성구분</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>AI 추정원인</t>
         </is>
       </c>
     </row>
@@ -620,6 +633,16 @@
           <t>일치</t>
         </is>
       </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>경미한 차이</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
@@ -682,6 +705,16 @@
           <t>불일치</t>
         </is>
       </c>
+      <c r="S3" s="4" t="inlineStr">
+        <is>
+          <t>경미한 차이</t>
+        </is>
+      </c>
+      <c r="T3" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -744,6 +777,16 @@
           <t>일치</t>
         </is>
       </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>경미한 차이</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -806,6 +849,16 @@
           <t>일치</t>
         </is>
       </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>경미한 차이</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -868,6 +921,16 @@
           <t>일치</t>
         </is>
       </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>경미한 차이</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -930,6 +993,16 @@
           <t>불일치</t>
         </is>
       </c>
+      <c r="S7" s="4" t="inlineStr">
+        <is>
+          <t>경미한 차이</t>
+        </is>
+      </c>
+      <c r="T7" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -992,6 +1065,16 @@
           <t>일치</t>
         </is>
       </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>경미한 차이</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1054,6 +1137,16 @@
           <t>일치</t>
         </is>
       </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>경미한 차이</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
@@ -1116,6 +1209,16 @@
           <t>불일치</t>
         </is>
       </c>
+      <c r="S10" s="4" t="inlineStr">
+        <is>
+          <t>경미한 차이</t>
+        </is>
+      </c>
+      <c r="T10" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1178,6 +1281,16 @@
           <t>일치</t>
         </is>
       </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>경미한 차이</t>
+        </is>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1242,6 +1355,16 @@
           <t>일치</t>
         </is>
       </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>경미한 차이</t>
+        </is>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1306,6 +1429,16 @@
       <c r="R13" t="inlineStr">
         <is>
           <t>일치</t>
+        </is>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>경미한 차이</t>
+        </is>
+      </c>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -1370,9 +1503,19 @@
           <t>일치</t>
         </is>
       </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>경미한 차이</t>
+        </is>
+      </c>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:R14"/>
+  <autoFilter ref="A1:T14"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1383,7 +1526,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R4"/>
+  <dimension ref="A1:T4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1404,6 +1547,8 @@
     <col width="15" customWidth="1" min="16" max="16"/>
     <col width="16" customWidth="1" min="17" max="17"/>
     <col width="14" customWidth="1" min="18" max="18"/>
+    <col width="14" customWidth="1" min="19" max="19"/>
+    <col width="60" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1495,6 +1640,16 @@
       <c r="R1" s="1" t="inlineStr">
         <is>
           <t>일치여부</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>중요성구분</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>AI 추정원인</t>
         </is>
       </c>
     </row>
@@ -1559,6 +1714,16 @@
           <t>불일치</t>
         </is>
       </c>
+      <c r="S2" s="4" t="inlineStr">
+        <is>
+          <t>경미한 차이</t>
+        </is>
+      </c>
+      <c r="T2" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
@@ -1621,6 +1786,16 @@
           <t>불일치</t>
         </is>
       </c>
+      <c r="S3" s="4" t="inlineStr">
+        <is>
+          <t>경미한 차이</t>
+        </is>
+      </c>
+      <c r="T3" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
@@ -1683,9 +1858,157 @@
           <t>불일치</t>
         </is>
       </c>
+      <c r="S4" s="4" t="inlineStr">
+        <is>
+          <t>경미한 차이</t>
+        </is>
+      </c>
+      <c r="T4" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:R4"/>
+  <autoFilter ref="A1:T4"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:T1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="16" customWidth="1" min="15" max="15"/>
+    <col width="15" customWidth="1" min="16" max="16"/>
+    <col width="16" customWidth="1" min="17" max="17"/>
+    <col width="14" customWidth="1" min="18" max="18"/>
+    <col width="14" customWidth="1" min="19" max="19"/>
+    <col width="60" customWidth="1" min="20" max="20"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>자산명</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>자산분류</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>취득일</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>취득원가</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>잔존가치</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>내용연수(년)</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>상각방법</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>처분일</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>내용연수재추정일</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>재추정후내용연수(년)</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>경과개월수(취득일~기준일)</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>당기해당월수</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>내용연수종료여부</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>비고</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>회사반영_당기감가상각비</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>재계산_당기감가상각비</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>차이(재계산-회사반영)</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>일치여부</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>중요성구분</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>AI 추정원인</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>